<commit_message>
Clean-up becomes optional step 3; brand guide PDF colors; standard vs custom category wording; schema registry workbook; study type options locked
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/orgs/dada2/overlay.xlsx
+++ b/orgs/dada2/overlay.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule additions" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Display groups" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Genes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom call groups" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -560,6 +561,57 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Call group</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sections sent to the AI (separate with ;)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>If those sections hold fewer than this many characters, send the whole paper</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Also send every section that starts on this page or earlier (0 = none)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Re-read the whole paper when a category is not found? (Always / Only if key sections are missing / Never)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Key sections (a re-read is skipped when the paper has any of these)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -608,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -768,6 +820,28 @@
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Clinical features observed in this paper's own patients (vasculitis, stroke, cytopenia, immunodeficiency, livedo, fever, and so on).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>study_type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>filter_chip</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>